<commit_message>
xử lý ngày nghỉ có phép
</commit_message>
<xml_diff>
--- a/convert/Cong_thang_4.xlsx
+++ b/convert/Cong_thang_4.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>2022-04-01</t>
   </si>
@@ -64,7 +64,7 @@
     <t>2021-04-07</t>
   </si>
   <si>
-    <t>P</t>
+    <t>Co don nhung di lam</t>
   </si>
   <si>
     <t>A</t>
@@ -80,9 +80,6 @@
   </si>
   <si>
     <t>P0</t>
-  </si>
-  <si>
-    <t>L</t>
   </si>
 </sst>
 </file>
@@ -493,7 +490,7 @@
         <v>21</v>
       </c>
       <c r="W8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="AA8" t="s">
         <v>21</v>

</xml_diff>